<commit_message>
feat: Attention Center — review rejected/flagged activities with approve/reject/dismiss
</commit_message>
<xml_diff>
--- a/Walkathon Nominations 2026_Final.xlsx
+++ b/Walkathon Nominations 2026_Final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/epxxvis/projects/walky/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B743D15-485E-FC47-803E-873F70C39BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC79A41-C506-BC49-9845-EDC7313BD705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet2!$A$1:$H$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet2!$A$1:$J$161</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="813">
   <si>
     <t>Team Name</t>
   </si>
@@ -1625,9 +1625,6 @@
   </si>
   <si>
     <t>Kamalakannan Sudhakar | Strava Athlete Profile</t>
-  </si>
-  <si>
-    <t>Unassigned</t>
   </si>
   <si>
     <t>ZMANRAO</t>
@@ -2930,6 +2927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J161"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2978,7 +2976,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -3010,7 +3008,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
@@ -3074,7 +3072,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
@@ -3106,7 +3104,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -3138,7 +3136,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -3170,7 +3168,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
@@ -3202,7 +3200,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -3234,7 +3232,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
@@ -3266,7 +3264,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -3298,7 +3296,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
@@ -3330,7 +3328,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>10</v>
       </c>
@@ -3362,7 +3360,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>10</v>
       </c>
@@ -3394,7 +3392,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>10</v>
       </c>
@@ -3490,7 +3488,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>10</v>
       </c>
@@ -3522,7 +3520,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
@@ -3554,7 +3552,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>10</v>
       </c>
@@ -3586,7 +3584,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>10</v>
       </c>
@@ -3618,7 +3616,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>114</v>
       </c>
@@ -3650,7 +3648,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>114</v>
       </c>
@@ -3682,7 +3680,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>114</v>
       </c>
@@ -3714,7 +3712,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>114</v>
       </c>
@@ -3746,7 +3744,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>114</v>
       </c>
@@ -3810,7 +3808,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>114</v>
       </c>
@@ -3842,7 +3840,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>114</v>
       </c>
@@ -3874,7 +3872,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>114</v>
       </c>
@@ -3906,7 +3904,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>114</v>
       </c>
@@ -3938,7 +3936,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>114</v>
       </c>
@@ -4002,7 +4000,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>114</v>
       </c>
@@ -4034,7 +4032,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>114</v>
       </c>
@@ -4066,7 +4064,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>114</v>
       </c>
@@ -4098,7 +4096,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>114</v>
       </c>
@@ -4130,7 +4128,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>114</v>
       </c>
@@ -4162,7 +4160,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>114</v>
       </c>
@@ -4226,7 +4224,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>114</v>
       </c>
@@ -4258,7 +4256,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>213</v>
       </c>
@@ -4322,7 +4320,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>213</v>
       </c>
@@ -4674,7 +4672,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="5" t="s">
         <v>213</v>
       </c>
@@ -4770,7 +4768,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
         <v>213</v>
       </c>
@@ -4930,7 +4928,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>312</v>
       </c>
@@ -5026,7 +5024,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>312</v>
       </c>
@@ -5090,7 +5088,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>312</v>
       </c>
@@ -5186,7 +5184,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>312</v>
       </c>
@@ -5314,7 +5312,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>312</v>
       </c>
@@ -5346,7 +5344,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>312</v>
       </c>
@@ -5506,7 +5504,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>312</v>
       </c>
@@ -5538,7 +5536,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>413</v>
       </c>
@@ -5570,7 +5568,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>413</v>
       </c>
@@ -5666,7 +5664,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>413</v>
       </c>
@@ -5698,7 +5696,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>413</v>
       </c>
@@ -5730,7 +5728,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>413</v>
       </c>
@@ -5762,7 +5760,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>413</v>
       </c>
@@ -5826,7 +5824,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>413</v>
       </c>
@@ -5890,7 +5888,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>413</v>
       </c>
@@ -5954,7 +5952,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>413</v>
       </c>
@@ -5986,7 +5984,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>413</v>
       </c>
@@ -6018,7 +6016,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>413</v>
       </c>
@@ -6050,7 +6048,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>413</v>
       </c>
@@ -6082,7 +6080,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>413</v>
       </c>
@@ -6178,7 +6176,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>514</v>
       </c>
@@ -6210,7 +6208,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>514</v>
       </c>
@@ -6242,7 +6240,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
         <v>514</v>
       </c>
@@ -6274,7 +6272,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>514</v>
       </c>
@@ -6303,33 +6301,33 @@
         <v>29</v>
       </c>
       <c r="J105" s="10" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B106" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C106" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="C106" s="2" t="s">
+      <c r="D106" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E106" s="8" t="s">
         <v>536</v>
-      </c>
-      <c r="D106" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E106" s="8" t="s">
-        <v>537</v>
       </c>
       <c r="F106" s="2">
         <v>9985541711</v>
       </c>
       <c r="G106" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="H106" s="10" t="s">
         <v>538</v>
-      </c>
-      <c r="H106" s="10" t="s">
-        <v>539</v>
       </c>
       <c r="I106" s="10" t="s">
         <v>17</v>
@@ -6343,25 +6341,25 @@
         <v>514</v>
       </c>
       <c r="B107" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="C107" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="C107" s="2" t="s">
+      <c r="D107" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E107" s="2" t="s">
         <v>541</v>
-      </c>
-      <c r="D107" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E107" s="2" t="s">
-        <v>542</v>
       </c>
       <c r="F107" s="2">
         <v>919841248577</v>
       </c>
       <c r="G107" s="7" t="s">
+        <v>542</v>
+      </c>
+      <c r="H107" s="10" t="s">
         <v>543</v>
-      </c>
-      <c r="H107" s="10" t="s">
-        <v>544</v>
       </c>
       <c r="I107" s="10" t="s">
         <v>29</v>
@@ -6370,30 +6368,30 @@
         <v>30</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B108" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="C108" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="C108" s="2" t="s">
+      <c r="D108" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E108" s="7" t="s">
         <v>546</v>
-      </c>
-      <c r="D108" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E108" s="7" t="s">
-        <v>547</v>
       </c>
       <c r="F108" s="2">
         <v>919500074227</v>
       </c>
       <c r="G108" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="H108" s="10" t="s">
         <v>548</v>
-      </c>
-      <c r="H108" s="10" t="s">
-        <v>549</v>
       </c>
       <c r="I108" s="10" t="s">
         <v>17</v>
@@ -6407,22 +6405,22 @@
         <v>514</v>
       </c>
       <c r="B109" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="C109" s="2" t="s">
+      <c r="D109" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E109" s="7" t="s">
         <v>551</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E109" s="7" t="s">
-        <v>552</v>
       </c>
       <c r="F109" s="2">
         <v>6382811325</v>
       </c>
       <c r="G109" s="7" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="H109" s="10">
         <v>1570233933</v>
@@ -6434,30 +6432,30 @@
         <v>30</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B110" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="C110" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C110" s="2" t="s">
+      <c r="D110" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E110" s="2" t="s">
         <v>555</v>
-      </c>
-      <c r="D110" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>556</v>
       </c>
       <c r="F110" s="2">
         <v>919600199456</v>
       </c>
       <c r="G110" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="H110" s="10" t="s">
         <v>557</v>
-      </c>
-      <c r="H110" s="10" t="s">
-        <v>558</v>
       </c>
       <c r="I110" s="10" t="s">
         <v>17</v>
@@ -6471,25 +6469,25 @@
         <v>514</v>
       </c>
       <c r="B111" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="C111" s="2" t="s">
         <v>559</v>
-      </c>
-      <c r="C111" s="2" t="s">
-        <v>560</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F111" s="2">
         <v>918939833531</v>
       </c>
       <c r="G111" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="H111" s="10" t="s">
         <v>562</v>
-      </c>
-      <c r="H111" s="10" t="s">
-        <v>563</v>
       </c>
       <c r="I111" s="10" t="s">
         <v>29</v>
@@ -6498,30 +6496,30 @@
         <v>30</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B112" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C112" s="2" t="s">
         <v>564</v>
-      </c>
-      <c r="C112" s="2" t="s">
-        <v>565</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E112" s="7" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F112" s="2">
         <v>9958777360</v>
       </c>
       <c r="G112" s="6" t="s">
+        <v>566</v>
+      </c>
+      <c r="H112" s="10" t="s">
         <v>567</v>
-      </c>
-      <c r="H112" s="10" t="s">
-        <v>568</v>
       </c>
       <c r="I112" s="10" t="s">
         <v>17</v>
@@ -6535,25 +6533,25 @@
         <v>514</v>
       </c>
       <c r="B113" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="C113" s="2" t="s">
         <v>569</v>
-      </c>
-      <c r="C113" s="2" t="s">
-        <v>570</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="F113" s="2">
         <v>9894916995</v>
       </c>
       <c r="G113" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="H113" s="10" t="s">
         <v>572</v>
-      </c>
-      <c r="H113" s="10" t="s">
-        <v>573</v>
       </c>
       <c r="I113" s="10" t="s">
         <v>29</v>
@@ -6562,30 +6560,30 @@
         <v>30</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B114" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="C114" s="2" t="s">
         <v>574</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>575</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F114" s="2">
         <v>9500043735</v>
       </c>
       <c r="G114" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="H114" s="10" t="s">
         <v>577</v>
-      </c>
-      <c r="H114" s="10" t="s">
-        <v>578</v>
       </c>
       <c r="I114" s="10" t="s">
         <v>17</v>
@@ -6599,25 +6597,25 @@
         <v>514</v>
       </c>
       <c r="B115" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="C115" s="2" t="s">
         <v>579</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>580</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E115" s="7" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="F115" s="2">
         <v>6369326376</v>
       </c>
       <c r="G115" s="7" t="s">
+        <v>581</v>
+      </c>
+      <c r="H115" s="10" t="s">
         <v>582</v>
-      </c>
-      <c r="H115" s="10" t="s">
-        <v>583</v>
       </c>
       <c r="I115" s="10" t="s">
         <v>29</v>
@@ -6626,31 +6624,31 @@
         <v>30</v>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B116" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C116" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="C116" s="2" t="s">
+      <c r="D116" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E116" s="2" t="s">
         <v>585</v>
-      </c>
-      <c r="D116" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>586</v>
       </c>
       <c r="F116" s="2">
         <v>9003724569</v>
       </c>
       <c r="G116" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="H116" s="10" t="s">
         <v>587</v>
       </c>
-      <c r="H116" s="10" t="s">
-        <v>588</v>
-      </c>
       <c r="I116" s="10" t="s">
         <v>17</v>
       </c>
@@ -6658,31 +6656,31 @@
         <v>18</v>
       </c>
     </row>
-    <row r="117" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B117" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="C117" s="2" t="s">
         <v>589</v>
       </c>
-      <c r="C117" s="2" t="s">
+      <c r="D117" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E117" s="7" t="s">
         <v>590</v>
-      </c>
-      <c r="D117" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E117" s="7" t="s">
-        <v>591</v>
       </c>
       <c r="F117" s="2">
         <v>9894540684</v>
       </c>
       <c r="G117" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="H117" s="10" t="s">
         <v>592</v>
       </c>
-      <c r="H117" s="10" t="s">
-        <v>593</v>
-      </c>
       <c r="I117" s="10" t="s">
         <v>17</v>
       </c>
@@ -6690,31 +6688,31 @@
         <v>18</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B118" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="C118" s="2" t="s">
+      <c r="D118" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E118" s="7" t="s">
         <v>595</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E118" s="7" t="s">
-        <v>596</v>
       </c>
       <c r="F118" s="2">
         <v>9789810530</v>
       </c>
       <c r="G118" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="H118" s="10" t="s">
         <v>597</v>
       </c>
-      <c r="H118" s="10" t="s">
-        <v>598</v>
-      </c>
       <c r="I118" s="10" t="s">
         <v>17</v>
       </c>
@@ -6722,31 +6720,31 @@
         <v>18</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B119" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="C119" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="C119" s="2" t="s">
+      <c r="D119" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E119" s="7" t="s">
         <v>600</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E119" s="7" t="s">
-        <v>601</v>
       </c>
       <c r="F119" s="2">
         <v>9551635956</v>
       </c>
       <c r="G119" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="H119" s="10" t="s">
         <v>602</v>
       </c>
-      <c r="H119" s="10" t="s">
-        <v>603</v>
-      </c>
       <c r="I119" s="10" t="s">
         <v>17</v>
       </c>
@@ -6754,30 +6752,30 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
         <v>514</v>
       </c>
       <c r="B120" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="C120" s="2" t="s">
         <v>604</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>605</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F120" s="2">
         <v>919884025540</v>
       </c>
       <c r="G120" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="H120" s="10" t="s">
         <v>607</v>
-      </c>
-      <c r="H120" s="10" t="s">
-        <v>608</v>
       </c>
       <c r="I120" s="10" t="s">
         <v>17</v>
@@ -6791,25 +6789,25 @@
         <v>514</v>
       </c>
       <c r="B121" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="C121" s="2" t="s">
         <v>609</v>
-      </c>
-      <c r="C121" s="2" t="s">
-        <v>610</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F121" s="2">
         <v>919677333273</v>
       </c>
       <c r="G121" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="H121" s="10" t="s">
         <v>612</v>
-      </c>
-      <c r="H121" s="10" t="s">
-        <v>613</v>
       </c>
       <c r="I121" s="10" t="s">
         <v>29</v>
@@ -6818,447 +6816,447 @@
         <v>30</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B122" s="2" t="s">
         <v>614</v>
       </c>
-      <c r="B122" s="2" t="s">
+      <c r="C122" s="2" t="s">
         <v>615</v>
       </c>
-      <c r="C122" s="2" t="s">
+      <c r="D122" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E122" s="2" t="s">
         <v>616</v>
-      </c>
-      <c r="D122" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E122" s="2" t="s">
-        <v>617</v>
       </c>
       <c r="F122" s="2">
         <v>8754129067</v>
       </c>
       <c r="G122" s="7" t="s">
+        <v>617</v>
+      </c>
+      <c r="H122" s="10" t="s">
         <v>618</v>
       </c>
-      <c r="H122" s="10" t="s">
+      <c r="I122" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J122" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A123" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B123" s="2" t="s">
         <v>619</v>
       </c>
-      <c r="I122" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J122" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B123" s="2" t="s">
+      <c r="C123" s="2" t="s">
         <v>620</v>
       </c>
-      <c r="C123" s="2" t="s">
+      <c r="D123" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E123" s="2" t="s">
         <v>621</v>
-      </c>
-      <c r="D123" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E123" s="2" t="s">
-        <v>622</v>
       </c>
       <c r="F123" s="2">
         <v>8144368800</v>
       </c>
       <c r="G123" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="H123" s="10" t="s">
         <v>623</v>
       </c>
-      <c r="H123" s="10" t="s">
+      <c r="I123" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J123" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A124" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B124" s="2" t="s">
         <v>624</v>
       </c>
-      <c r="I123" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J123" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B124" s="2" t="s">
+      <c r="C124" s="2" t="s">
         <v>625</v>
       </c>
-      <c r="C124" s="2" t="s">
+      <c r="D124" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E124" s="2" t="s">
         <v>626</v>
-      </c>
-      <c r="D124" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E124" s="2" t="s">
-        <v>627</v>
       </c>
       <c r="F124" s="2">
         <v>9842756727</v>
       </c>
       <c r="G124" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="H124" s="10" t="s">
         <v>628</v>
       </c>
-      <c r="H124" s="10" t="s">
+      <c r="I124" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J124" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A125" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B125" s="2" t="s">
         <v>629</v>
       </c>
-      <c r="I124" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J124" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B125" s="2" t="s">
+      <c r="C125" s="2" t="s">
         <v>630</v>
-      </c>
-      <c r="C125" s="2" t="s">
-        <v>631</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F125" s="2">
         <v>9488833626</v>
       </c>
       <c r="G125" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="H125" s="10" t="s">
         <v>633</v>
       </c>
-      <c r="H125" s="10" t="s">
+      <c r="I125" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J125" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A126" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B126" s="2" t="s">
         <v>634</v>
       </c>
-      <c r="I125" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J125" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B126" s="2" t="s">
+      <c r="C126" s="2" t="s">
         <v>635</v>
       </c>
-      <c r="C126" s="2" t="s">
+      <c r="D126" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E126" s="2" t="s">
         <v>636</v>
-      </c>
-      <c r="D126" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E126" s="2" t="s">
-        <v>637</v>
       </c>
       <c r="F126" s="2">
         <v>7382432136</v>
       </c>
       <c r="G126" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="H126" s="10" t="s">
         <v>638</v>
       </c>
-      <c r="H126" s="10" t="s">
+      <c r="I126" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J126" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A127" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B127" s="2" t="s">
         <v>639</v>
       </c>
-      <c r="I126" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J126" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B127" s="2" t="s">
+      <c r="C127" s="2" t="s">
         <v>640</v>
       </c>
-      <c r="C127" s="2" t="s">
+      <c r="D127" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E127" s="2" t="s">
         <v>641</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>642</v>
       </c>
       <c r="F127" s="2">
         <v>9842956552</v>
       </c>
       <c r="G127" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="H127" s="10" t="s">
         <v>643</v>
       </c>
-      <c r="H127" s="10" t="s">
+      <c r="I127" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J127" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A128" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B128" s="2" t="s">
         <v>644</v>
       </c>
-      <c r="I127" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J127" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B128" s="2" t="s">
+      <c r="C128" s="2" t="s">
         <v>645</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>646</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="F128" s="2">
         <v>9790998583</v>
       </c>
       <c r="G128" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="H128" s="10" t="s">
         <v>648</v>
       </c>
-      <c r="H128" s="10" t="s">
+      <c r="I128" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J128" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A129" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B129" s="2" t="s">
         <v>649</v>
       </c>
-      <c r="I128" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J128" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B129" s="2" t="s">
+      <c r="C129" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C129" s="2" t="s">
+      <c r="D129" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E129" s="2" t="s">
         <v>651</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E129" s="2" t="s">
-        <v>652</v>
       </c>
       <c r="F129" s="2">
         <v>9123521909</v>
       </c>
       <c r="G129" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="H129" s="10" t="s">
         <v>653</v>
       </c>
-      <c r="H129" s="10" t="s">
+      <c r="I129" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J129" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B130" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="I129" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J129" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B130" s="2" t="s">
+      <c r="C130" s="2" t="s">
         <v>655</v>
       </c>
-      <c r="C130" s="2" t="s">
+      <c r="D130" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E130" s="2" t="s">
         <v>656</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>657</v>
       </c>
       <c r="F130" s="2">
         <v>9790909930</v>
       </c>
       <c r="G130" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="H130" s="10" t="s">
         <v>658</v>
       </c>
-      <c r="H130" s="10" t="s">
+      <c r="I130" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J130" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B131" s="2" t="s">
         <v>659</v>
       </c>
-      <c r="I130" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J130" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B131" s="2" t="s">
+      <c r="C131" s="2" t="s">
         <v>660</v>
       </c>
-      <c r="C131" s="2" t="s">
+      <c r="D131" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E131" s="2" t="s">
         <v>661</v>
-      </c>
-      <c r="D131" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E131" s="2" t="s">
-        <v>662</v>
       </c>
       <c r="F131" s="2">
         <v>9843451933</v>
       </c>
       <c r="G131" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="H131" s="10" t="s">
         <v>663</v>
       </c>
-      <c r="H131" s="10" t="s">
+      <c r="I131" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J131" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B132" s="2" t="s">
         <v>664</v>
       </c>
-      <c r="I131" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J131" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B132" s="2" t="s">
+      <c r="C132" s="2" t="s">
         <v>665</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="D132" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E132" s="2" t="s">
         <v>666</v>
-      </c>
-      <c r="D132" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E132" s="2" t="s">
-        <v>667</v>
       </c>
       <c r="F132" s="2">
         <v>9940182025</v>
       </c>
       <c r="G132" s="7" t="s">
+        <v>667</v>
+      </c>
+      <c r="H132" s="10" t="s">
         <v>668</v>
       </c>
-      <c r="H132" s="10" t="s">
+      <c r="I132" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J132" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B133" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="I132" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J132" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B133" s="2" t="s">
+      <c r="C133" s="2" t="s">
         <v>670</v>
-      </c>
-      <c r="C133" s="2" t="s">
-        <v>671</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F133" s="2">
         <v>9092487649</v>
       </c>
       <c r="G133" s="7" t="s">
+        <v>672</v>
+      </c>
+      <c r="H133" s="10" t="s">
         <v>673</v>
       </c>
-      <c r="H133" s="10" t="s">
+      <c r="I133" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J133" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B134" s="2" t="s">
         <v>674</v>
       </c>
-      <c r="I133" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J133" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B134" s="2" t="s">
+      <c r="C134" s="2" t="s">
         <v>675</v>
       </c>
-      <c r="C134" s="2" t="s">
+      <c r="D134" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E134" s="2" t="s">
         <v>676</v>
-      </c>
-      <c r="D134" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E134" s="2" t="s">
-        <v>677</v>
       </c>
       <c r="F134" s="2">
         <v>9900487944</v>
       </c>
       <c r="G134" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="H134" s="10" t="s">
         <v>678</v>
       </c>
-      <c r="H134" s="10" t="s">
+      <c r="I134" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J134" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B135" s="2" t="s">
         <v>679</v>
       </c>
-      <c r="I134" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J134" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B135" s="2" t="s">
+      <c r="C135" s="2" t="s">
         <v>680</v>
       </c>
-      <c r="C135" s="2" t="s">
+      <c r="D135" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E135" s="2" t="s">
         <v>681</v>
-      </c>
-      <c r="D135" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E135" s="2" t="s">
-        <v>682</v>
       </c>
       <c r="F135" s="2">
         <v>9751234404</v>
       </c>
       <c r="G135" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="H135" s="10" t="s">
         <v>623</v>
       </c>
-      <c r="H135" s="10" t="s">
-        <v>624</v>
-      </c>
       <c r="I135" s="10" t="s">
         <v>17</v>
       </c>
@@ -7266,414 +7264,414 @@
         <v>18</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B136" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="C136" s="2" t="s">
         <v>683</v>
       </c>
-      <c r="C136" s="2" t="s">
+      <c r="D136" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E136" s="2" t="s">
         <v>684</v>
-      </c>
-      <c r="D136" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E136" s="2" t="s">
-        <v>685</v>
       </c>
       <c r="F136" s="2">
         <v>9944194100</v>
       </c>
       <c r="G136" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="H136" s="10" t="s">
         <v>686</v>
       </c>
-      <c r="H136" s="10" t="s">
+      <c r="I136" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J136" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B137" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="I136" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J136" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B137" s="2" t="s">
+      <c r="C137" s="2" t="s">
         <v>688</v>
-      </c>
-      <c r="C137" s="2" t="s">
-        <v>689</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="F137" s="2">
         <v>6361759520</v>
       </c>
       <c r="G137" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="H137" s="10" t="s">
         <v>691</v>
       </c>
-      <c r="H137" s="10" t="s">
+      <c r="I137" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J137" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A138" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B138" s="2" t="s">
         <v>692</v>
       </c>
-      <c r="I137" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J137" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B138" s="2" t="s">
+      <c r="C138" s="2" t="s">
         <v>693</v>
       </c>
-      <c r="C138" s="2" t="s">
+      <c r="D138" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E138" s="2" t="s">
         <v>694</v>
-      </c>
-      <c r="D138" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E138" s="2" t="s">
-        <v>695</v>
       </c>
       <c r="F138" s="2">
         <v>8376014306</v>
       </c>
       <c r="G138" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="H138" s="10" t="s">
         <v>696</v>
       </c>
-      <c r="H138" s="10" t="s">
+      <c r="I138" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J138" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A139" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B139" s="2" t="s">
         <v>697</v>
       </c>
-      <c r="I138" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J138" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B139" s="2" t="s">
+      <c r="C139" s="2" t="s">
         <v>698</v>
-      </c>
-      <c r="C139" s="2" t="s">
-        <v>699</v>
       </c>
       <c r="D139" s="5" t="s">
         <v>76</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="F139" s="2">
         <v>9790766914</v>
       </c>
       <c r="G139" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="H139" s="10" t="s">
         <v>701</v>
       </c>
-      <c r="H139" s="10" t="s">
+      <c r="I139" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J139" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A140" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B140" s="2" t="s">
         <v>702</v>
       </c>
-      <c r="I139" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J139" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B140" s="2" t="s">
+      <c r="C140" s="2" t="s">
         <v>703</v>
       </c>
-      <c r="C140" s="2" t="s">
+      <c r="D140" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E140" s="2" t="s">
         <v>704</v>
-      </c>
-      <c r="D140" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E140" s="2" t="s">
-        <v>705</v>
       </c>
       <c r="F140" s="2">
         <v>9841255581</v>
       </c>
       <c r="G140" s="7" t="s">
+        <v>705</v>
+      </c>
+      <c r="H140" s="10" t="s">
         <v>706</v>
       </c>
-      <c r="H140" s="10" t="s">
+      <c r="I140" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J140" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A141" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B141" s="2" t="s">
         <v>707</v>
       </c>
-      <c r="I140" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J140" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="B141" s="2" t="s">
+      <c r="C141" s="2" t="s">
         <v>708</v>
       </c>
-      <c r="C141" s="2" t="s">
+      <c r="D141" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E141" s="2" t="s">
         <v>709</v>
-      </c>
-      <c r="D141" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E141" s="2" t="s">
-        <v>710</v>
       </c>
       <c r="F141" s="2">
         <v>9843451933</v>
       </c>
       <c r="G141" s="7" t="s">
+        <v>710</v>
+      </c>
+      <c r="H141" s="10" t="s">
         <v>711</v>
       </c>
-      <c r="H141" s="10" t="s">
+      <c r="I141" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J141" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" s="2" t="s">
         <v>712</v>
       </c>
-      <c r="I141" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J141" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A142" s="2" t="s">
+      <c r="B142" s="2" t="s">
         <v>713</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="C142" s="2" t="s">
         <v>714</v>
       </c>
-      <c r="C142" s="2" t="s">
+      <c r="D142" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E142" s="2" t="s">
         <v>715</v>
-      </c>
-      <c r="D142" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E142" s="2" t="s">
-        <v>716</v>
       </c>
       <c r="F142" s="2">
         <v>8754425672</v>
       </c>
       <c r="G142" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="H142" s="10" t="s">
         <v>717</v>
       </c>
-      <c r="H142" s="10" t="s">
+      <c r="I142" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J142" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B143" s="2" t="s">
         <v>718</v>
       </c>
-      <c r="I142" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J142" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B143" s="2" t="s">
+      <c r="C143" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="C143" s="2" t="s">
+      <c r="D143" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E143" s="2" t="s">
         <v>720</v>
-      </c>
-      <c r="D143" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E143" s="2" t="s">
-        <v>721</v>
       </c>
       <c r="F143" s="2">
         <v>7397271607</v>
       </c>
       <c r="G143" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="H143" s="10" t="s">
         <v>722</v>
       </c>
-      <c r="H143" s="10" t="s">
+      <c r="I143" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J143" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B144" s="2" t="s">
         <v>723</v>
       </c>
-      <c r="I143" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J143" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="144" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B144" s="2" t="s">
+      <c r="C144" s="2" t="s">
         <v>724</v>
       </c>
-      <c r="C144" s="2" t="s">
+      <c r="D144" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E144" s="2" t="s">
         <v>725</v>
-      </c>
-      <c r="D144" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E144" s="2" t="s">
-        <v>726</v>
       </c>
       <c r="F144" s="2">
         <v>9940085134</v>
       </c>
       <c r="G144" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="H144" s="10" t="s">
         <v>727</v>
       </c>
-      <c r="H144" s="10" t="s">
+      <c r="I144" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J144" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B145" s="2" t="s">
         <v>728</v>
       </c>
-      <c r="I144" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J144" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="145" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B145" s="2" t="s">
+      <c r="C145" s="2" t="s">
         <v>729</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="D145" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E145" s="2" t="s">
         <v>730</v>
-      </c>
-      <c r="D145" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E145" s="2" t="s">
-        <v>731</v>
       </c>
       <c r="F145" s="2">
         <v>9528537800</v>
       </c>
       <c r="G145" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="H145" s="10" t="s">
         <v>732</v>
       </c>
-      <c r="H145" s="10" t="s">
+      <c r="I145" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J145" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B146" s="2" t="s">
         <v>733</v>
       </c>
-      <c r="I145" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J145" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="146" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B146" s="2" t="s">
+      <c r="C146" s="2" t="s">
         <v>734</v>
       </c>
-      <c r="C146" s="2" t="s">
+      <c r="D146" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E146" s="2" t="s">
         <v>735</v>
-      </c>
-      <c r="D146" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>736</v>
       </c>
       <c r="F146" s="2">
         <v>8438234525</v>
       </c>
       <c r="G146" s="7" t="s">
+        <v>736</v>
+      </c>
+      <c r="H146" s="10" t="s">
         <v>737</v>
       </c>
-      <c r="H146" s="10" t="s">
+      <c r="I146" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J146" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B147" s="2" t="s">
         <v>738</v>
       </c>
-      <c r="I146" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J146" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="147" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B147" s="2" t="s">
+      <c r="C147" s="2" t="s">
         <v>739</v>
       </c>
-      <c r="C147" s="2" t="s">
+      <c r="D147" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E147" s="2" t="s">
         <v>740</v>
-      </c>
-      <c r="D147" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E147" s="2" t="s">
-        <v>741</v>
       </c>
       <c r="F147" s="2">
         <v>9566029509</v>
       </c>
       <c r="G147" s="7" t="s">
+        <v>741</v>
+      </c>
+      <c r="H147" s="10" t="s">
         <v>742</v>
       </c>
-      <c r="H147" s="10" t="s">
+      <c r="I147" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J147" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B148" s="2" t="s">
         <v>743</v>
       </c>
-      <c r="I147" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J147" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="148" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B148" s="2" t="s">
+      <c r="C148" s="2" t="s">
         <v>744</v>
       </c>
-      <c r="C148" s="2" t="s">
+      <c r="D148" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E148" s="2" t="s">
         <v>745</v>
-      </c>
-      <c r="D148" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E148" s="2" t="s">
-        <v>746</v>
       </c>
       <c r="F148" s="2">
         <v>9941014154</v>
       </c>
       <c r="G148" s="7" t="s">
+        <v>746</v>
+      </c>
+      <c r="H148" s="10" t="s">
         <v>747</v>
-      </c>
-      <c r="H148" s="10" t="s">
-        <v>748</v>
       </c>
       <c r="I148" s="10" t="s">
         <v>17</v>
@@ -7684,28 +7682,28 @@
     </row>
     <row r="149" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B149" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="C149" s="2" t="s">
         <v>749</v>
       </c>
-      <c r="C149" s="2" t="s">
+      <c r="D149" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E149" s="2" t="s">
         <v>750</v>
-      </c>
-      <c r="D149" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E149" s="2" t="s">
-        <v>751</v>
       </c>
       <c r="F149" s="2">
         <v>9176404337</v>
       </c>
       <c r="G149" s="7" t="s">
+        <v>751</v>
+      </c>
+      <c r="H149" s="10" t="s">
         <v>752</v>
-      </c>
-      <c r="H149" s="10" t="s">
-        <v>753</v>
       </c>
       <c r="I149" s="10" t="s">
         <v>29</v>
@@ -7714,254 +7712,254 @@
         <v>30</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B150" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="C150" s="2" t="s">
         <v>754</v>
       </c>
-      <c r="C150" s="2" t="s">
+      <c r="D150" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E150" s="2" t="s">
         <v>755</v>
-      </c>
-      <c r="D150" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>756</v>
       </c>
       <c r="F150" s="2">
         <v>7780198696</v>
       </c>
       <c r="G150" s="7" t="s">
+        <v>756</v>
+      </c>
+      <c r="H150" s="10" t="s">
         <v>757</v>
       </c>
-      <c r="H150" s="10" t="s">
+      <c r="I150" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J150" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A151" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B151" s="2" t="s">
         <v>758</v>
       </c>
-      <c r="I150" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J150" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="151" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B151" s="2" t="s">
+      <c r="C151" s="2" t="s">
         <v>759</v>
       </c>
-      <c r="C151" s="2" t="s">
+      <c r="D151" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E151" s="2" t="s">
         <v>760</v>
-      </c>
-      <c r="D151" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E151" s="2" t="s">
-        <v>761</v>
       </c>
       <c r="F151" s="2">
         <v>9094741005</v>
       </c>
       <c r="G151" s="7" t="s">
+        <v>761</v>
+      </c>
+      <c r="H151" s="10" t="s">
         <v>762</v>
       </c>
-      <c r="H151" s="10" t="s">
+      <c r="I151" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J151" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A152" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B152" s="2" t="s">
         <v>763</v>
       </c>
-      <c r="I151" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J151" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="152" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B152" s="2" t="s">
+      <c r="C152" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="C152" s="2" t="s">
+      <c r="D152" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E152" s="2" t="s">
         <v>765</v>
-      </c>
-      <c r="D152" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>766</v>
       </c>
       <c r="F152" s="2">
         <v>9884020052</v>
       </c>
       <c r="G152" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="H152" s="10" t="s">
         <v>767</v>
       </c>
-      <c r="H152" s="10" t="s">
+      <c r="I152" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J152" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A153" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B153" s="2" t="s">
         <v>768</v>
       </c>
-      <c r="I152" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J152" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="153" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B153" s="2" t="s">
+      <c r="C153" s="2" t="s">
         <v>769</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>770</v>
       </c>
       <c r="D153" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="F153" s="2">
         <v>8148182630</v>
       </c>
       <c r="G153" s="7" t="s">
+        <v>771</v>
+      </c>
+      <c r="H153" s="10" t="s">
         <v>772</v>
       </c>
-      <c r="H153" s="10" t="s">
+      <c r="I153" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J153" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A154" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B154" s="2" t="s">
         <v>773</v>
       </c>
-      <c r="I153" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J153" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="154" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B154" s="2" t="s">
+      <c r="C154" s="2" t="s">
         <v>774</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>775</v>
       </c>
       <c r="D154" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="F154" s="2">
         <v>7871171706</v>
       </c>
       <c r="G154" s="7" t="s">
+        <v>776</v>
+      </c>
+      <c r="H154" s="10" t="s">
         <v>777</v>
       </c>
-      <c r="H154" s="10" t="s">
+      <c r="I154" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J154" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A155" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B155" s="2" t="s">
         <v>778</v>
       </c>
-      <c r="I154" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J154" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="155" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B155" s="2" t="s">
+      <c r="C155" s="2" t="s">
         <v>779</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>780</v>
       </c>
       <c r="D155" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="F155" s="2">
         <v>8754412114</v>
       </c>
       <c r="G155" s="7" t="s">
+        <v>781</v>
+      </c>
+      <c r="H155" s="10" t="s">
         <v>782</v>
       </c>
-      <c r="H155" s="10" t="s">
+      <c r="I155" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J155" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A156" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B156" s="2" t="s">
         <v>783</v>
       </c>
-      <c r="I155" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J155" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="156" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B156" s="2" t="s">
+      <c r="C156" s="2" t="s">
         <v>784</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>785</v>
       </c>
       <c r="D156" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E156" s="2" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="F156" s="2">
         <v>9677025777</v>
       </c>
       <c r="G156" s="7" t="s">
+        <v>786</v>
+      </c>
+      <c r="H156" s="10" t="s">
         <v>787</v>
       </c>
-      <c r="H156" s="10" t="s">
+      <c r="I156" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J156" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A157" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="B157" s="2" t="s">
         <v>788</v>
       </c>
-      <c r="I156" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J156" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="157" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B157" s="2" t="s">
+      <c r="C157" s="2" t="s">
         <v>789</v>
-      </c>
-      <c r="C157" s="2" t="s">
-        <v>790</v>
       </c>
       <c r="D157" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="F157" s="2">
         <v>9486326998</v>
       </c>
       <c r="G157" s="7" t="s">
+        <v>791</v>
+      </c>
+      <c r="H157" s="10" t="s">
         <v>792</v>
-      </c>
-      <c r="H157" s="10" t="s">
-        <v>793</v>
       </c>
       <c r="I157" s="10" t="s">
         <v>17</v>
@@ -7972,28 +7970,28 @@
     </row>
     <row r="158" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B158" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="C158" s="2" t="s">
         <v>794</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>795</v>
       </c>
       <c r="D158" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="F158" s="2">
         <v>9790931473</v>
       </c>
       <c r="G158" s="7" t="s">
+        <v>796</v>
+      </c>
+      <c r="H158" s="10" t="s">
         <v>797</v>
-      </c>
-      <c r="H158" s="10" t="s">
-        <v>798</v>
       </c>
       <c r="I158" s="10" t="s">
         <v>29</v>
@@ -8004,28 +8002,28 @@
     </row>
     <row r="159" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B159" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="C159" s="2" t="s">
         <v>799</v>
       </c>
-      <c r="C159" s="2" t="s">
+      <c r="D159" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E159" s="2" t="s">
         <v>800</v>
-      </c>
-      <c r="D159" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E159" s="2" t="s">
-        <v>801</v>
       </c>
       <c r="F159" s="2">
         <v>9962573944</v>
       </c>
       <c r="G159" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="H159" s="10" t="s">
         <v>802</v>
-      </c>
-      <c r="H159" s="10" t="s">
-        <v>803</v>
       </c>
       <c r="I159" s="10" t="s">
         <v>29</v>
@@ -8036,28 +8034,28 @@
     </row>
     <row r="160" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B160" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="C160" s="2" t="s">
         <v>804</v>
       </c>
-      <c r="C160" s="2" t="s">
+      <c r="D160" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E160" s="2" t="s">
         <v>805</v>
-      </c>
-      <c r="D160" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E160" s="2" t="s">
-        <v>806</v>
       </c>
       <c r="F160" s="2">
         <v>9307444445</v>
       </c>
       <c r="G160" s="7" t="s">
+        <v>806</v>
+      </c>
+      <c r="H160" s="10" t="s">
         <v>807</v>
-      </c>
-      <c r="H160" s="10" t="s">
-        <v>808</v>
       </c>
       <c r="I160" s="10" t="s">
         <v>29</v>
@@ -8066,31 +8064,31 @@
         <v>30</v>
       </c>
     </row>
-    <row r="161" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:10" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B161" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="C161" s="2" t="s">
         <v>809</v>
       </c>
-      <c r="C161" s="2" t="s">
+      <c r="D161" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E161" s="2" t="s">
         <v>810</v>
-      </c>
-      <c r="D161" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E161" s="2" t="s">
-        <v>811</v>
       </c>
       <c r="F161" s="2">
         <v>8667742498</v>
       </c>
       <c r="G161" s="7" t="s">
+        <v>811</v>
+      </c>
+      <c r="H161" s="10" t="s">
         <v>812</v>
       </c>
-      <c r="H161" s="10" t="s">
-        <v>813</v>
-      </c>
       <c r="I161" s="10" t="s">
         <v>17</v>
       </c>
@@ -8099,6 +8097,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J161" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="Not Logged In"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D42:D55 D57:D59 D61 D122:D156 E157:E161" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Male,Female"</formula1>

</xml_diff>

<commit_message>
fix: PlayerDashboard uses viewAs context, overlay shows correctly in admin player preview
</commit_message>
<xml_diff>
--- a/Walkathon Nominations 2026_Final.xlsx
+++ b/Walkathon Nominations 2026_Final.xlsx
@@ -3014,7 +3014,7 @@
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>Not Logged In</t>
+          <t>Assigned</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
-          <t>Not Logged In</t>
+          <t>Assigned</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="J53" s="10" t="inlineStr">
         <is>
-          <t>Not Logged In</t>
+          <t>Assigned</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="J60" s="10" t="inlineStr">
         <is>
-          <t>Not Logged In</t>
+          <t>Assigned</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">

</xml_diff>

<commit_message>
fix: clear player selection after sync completes
</commit_message>
<xml_diff>
--- a/Walkathon Nominations 2026_Final.xlsx
+++ b/Walkathon Nominations 2026_Final.xlsx
@@ -3780,7 +3780,7 @@
       </c>
       <c r="J59" s="10" t="inlineStr">
         <is>
-          <t>Not Logged In</t>
+          <t>Assigned</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="J160" s="10" t="inlineStr">
         <is>
-          <t>Not Logged In</t>
+          <t>Assigned</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">

</xml_diff>